<commit_message>
Environment panel: headroom in stops with ≈× SDR white; trim monitor labels
The two-monitor test settled the unit from Chromium's source:
ScreenDetailed::hdrHeadroom() = log2(max(peak / SDR white, 1)). Show it as
"1.35 stops (≈2.55× SDR white)" instead of a raw number, and replace the
"unit not standardised" note with the unit plus the measured Windows caveat:
ScreenWin re-reads the SDR white level only on display-change, app-activation,
work-area, colour-profile or DXGI events, so brightness keys leave it stale.

Windows pads some monitor labels ("H32T13 "); readScreen now trims, and an
all-space label counts as none.

env_headroom_raw rewritten and env_headroom_value added in all 12 locales;
workbooks regenerated. check-display-watcher 63/63 (label trim, headroomRatio
against the user's measured 0.97/1.35/1.55); headless wiring run 20/20.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KyeyuyKaCpLNbSR2GQQh3Q
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B529"/>
+  <dimension ref="A1:B530"/>
   <cols>
     <col min="1" max="1" width="50.83203125" customWidth="1"/>
     <col min="2" max="2" width="50.83203125" customWidth="1"/>
@@ -3779,871 +3779,879 @@
     </row>
     <row r="422">
       <c r="A422" t="str">
-        <v>Shown exactly as the browser reports it. The unit is not standardised yet; an SDR screen has been observed to report 0.</v>
+        <v>Chromium reports this in stops: log₂ of the display’s peak brightness ÷ its SDR white level. On Windows it refreshes only when Chrome re-reads the display — the window moves to another screen, or Chrome becomes the active app again — not when brightness changes.</v>
       </c>
       <c r="B422" t="str">
-        <v>Genau so angezeigt, wie der Browser ihn meldet. Die Einheit ist noch nicht standardisiert; ein SDR-Bildschirm meldete 0.</v>
+        <v>Chromium meldet dies in Blendenstufen: log₂ aus Spitzenhelligkeit des Displays ÷ SDR-Weißpegel. Unter Windows wird der Wert nur aktualisiert, wenn Chrome das Display neu einliest – Fenster auf einen anderen Bildschirm verschoben oder Chrome wieder aktiviert –, nicht bei Helligkeitsänderungen.</v>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="str">
-        <v>HDR, gamut and pixel ratio refresh when the window moves to a screen where they differ.</v>
+        <v>{stops} stops (≈{ratio}× SDR white)</v>
       </c>
       <c r="B423" t="str">
-        <v>HDR, Farbraum und Pixelverhältnis werden aktualisiert, wenn das Fenster auf einen Bildschirm wechselt, auf dem sie abweichen.</v>
+        <v>{stops} Blendenstufen (≈{ratio}× SDR-Weiß)</v>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="str">
-        <v>Identify displays</v>
+        <v>HDR, gamut and pixel ratio refresh when the window moves to a screen where they differ.</v>
       </c>
       <c r="B424" t="str">
-        <v>Displays erkennen</v>
+        <v>HDR, Farbraum und Pixelverhältnis werden aktualisiert, wenn das Fenster auf einen Bildschirm wechselt, auf dem sie abweichen.</v>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="str">
-        <v>Asks permission to see which monitor this window is on, so the panel also refreshes when two screens look alike, and shows HDR headroom where the browser exposes it.</v>
+        <v>Identify displays</v>
       </c>
       <c r="B425" t="str">
-        <v>Fragt die Erlaubnis, zu sehen, auf welchem Monitor dieses Fenster liegt – so aktualisiert sich das Panel auch zwischen gleich wirkenden Bildschirmen und zeigt den HDR-Spielraum, wo der Browser ihn bereitstellt.</v>
+        <v>Displays erkennen</v>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="str">
-        <v>Tracking which monitor this window is on.</v>
+        <v>Asks permission to see which monitor this window is on, so the panel also refreshes when two screens look alike, and shows HDR headroom where the browser exposes it.</v>
       </c>
       <c r="B426" t="str">
-        <v>Verfolgt, auf welchem Monitor dieses Fenster liegt.</v>
+        <v>Fragt die Erlaubnis, zu sehen, auf welchem Monitor dieses Fenster liegt – so aktualisiert sich das Panel auch zwischen gleich wirkenden Bildschirmen und zeigt den HDR-Spielraum, wo der Browser ihn bereitstellt.</v>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="str">
-        <v>Permission to identify displays was refused. It can be changed in this site’s settings.</v>
+        <v>Tracking which monitor this window is on.</v>
       </c>
       <c r="B427" t="str">
-        <v>Die Erlaubnis zum Erkennen der Displays wurde verweigert. Sie lässt sich in den Einstellungen dieser Website ändern.</v>
+        <v>Verfolgt, auf welchem Monitor dieses Fenster liegt.</v>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="str">
-        <v>This browser cannot identify displays; only the automatic refresh above applies.</v>
+        <v>Permission to identify displays was refused. It can be changed in this site’s settings.</v>
       </c>
       <c r="B428" t="str">
-        <v>Dieser Browser kann Displays nicht erkennen; es gilt nur die automatische Aktualisierung oben.</v>
+        <v>Die Erlaubnis zum Erkennen der Displays wurde verweigert. Sie lässt sich in den Einstellungen dieser Website ändern.</v>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="str">
-        <v>Could not identify displays.</v>
+        <v>This browser cannot identify displays; only the automatic refresh above applies.</v>
       </c>
       <c r="B429" t="str">
-        <v>Displays konnten nicht erkannt werden.</v>
+        <v>Dieser Browser kann Displays nicht erkennen; es gilt nur die automatische Aktualisierung oben.</v>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="str">
-        <v>Display events</v>
+        <v>Could not identify displays.</v>
       </c>
       <c r="B430" t="str">
-        <v>Display-Ereignisse</v>
+        <v>Displays konnten nicht erkannt werden.</v>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="str">
-        <v>No events yet. Drag the window to another monitor.</v>
+        <v>Display events</v>
       </c>
       <c r="B431" t="str">
-        <v>Noch keine Ereignisse. Ziehen Sie das Fenster auf einen anderen Monitor.</v>
+        <v>Display-Ereignisse</v>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="str">
-        <v>Colour primaries</v>
+        <v>No events yet. Drag the window to another monitor.</v>
       </c>
       <c r="B432" t="str">
-        <v>Farbprimärvalenzen</v>
+        <v>Noch keine Ereignisse. Ziehen Sie das Fenster auf einen anderen Monitor.</v>
       </c>
     </row>
     <row r="433">
       <c r="A433" t="str">
-        <v>Transfer characteristics</v>
+        <v>Colour primaries</v>
       </c>
       <c r="B433" t="str">
-        <v>Übertragungsfunktion</v>
+        <v>Farbprimärvalenzen</v>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="str">
-        <v>Matrix coefficients</v>
+        <v>Transfer characteristics</v>
       </c>
       <c r="B434" t="str">
-        <v>Matrixkoeffizienten</v>
+        <v>Übertragungsfunktion</v>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="str">
-        <v>Video full-range flag</v>
+        <v>Matrix coefficients</v>
       </c>
       <c r="B435" t="str">
-        <v>Video-Vollbereichs-Flag</v>
+        <v>Matrixkoeffizienten</v>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="str">
-        <v>Full range</v>
+        <v>Video full-range flag</v>
       </c>
       <c r="B436" t="str">
-        <v>Vollbereich</v>
+        <v>Video-Vollbereichs-Flag</v>
       </c>
     </row>
     <row r="437">
       <c r="A437" t="str">
-        <v>Narrow range</v>
+        <v>Full range</v>
       </c>
       <c r="B437" t="str">
-        <v>Eingeschränkter Bereich</v>
+        <v>Vollbereich</v>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="str">
-        <v>not assigned by ITU-T H.273</v>
+        <v>Narrow range</v>
       </c>
       <c r="B438" t="str">
-        <v>von ITU-T H.273 nicht vergeben</v>
+        <v>Eingeschränkter Bereich</v>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="str">
-        <v>Colour primaries 2 (Unspecified) defers the primaries to the profile itself — they are taken from the colorant tags rather than from this tag.</v>
+        <v>not assigned by ITU-T H.273</v>
       </c>
       <c r="B439" t="str">
-        <v>Farbprimärvalenzen 2 (Nicht spezifiziert) verweist auf das Profil selbst — die Primärvalenzen stammen aus den Farbmittel-Tags, nicht aus diesem Tag.</v>
+        <v>von ITU-T H.273 nicht vergeben</v>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="str">
-        <v>The four reserved bytes of this tag are not all zero.</v>
+        <v>Colour primaries 2 (Unspecified) defers the primaries to the profile itself — they are taken from the colorant tags rather than from this tag.</v>
       </c>
       <c r="B440" t="str">
-        <v>Die vier reservierten Bytes dieses Tags sind nicht alle null.</v>
+        <v>Farbprimärvalenzen 2 (Nicht spezifiziert) verweist auf das Profil selbst — die Primärvalenzen stammen aus den Farbmittel-Tags, nicht aus diesem Tag.</v>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="str">
-        <v>REPORT</v>
+        <v>The four reserved bytes of this tag are not all zero.</v>
       </c>
       <c r="B441" t="str">
-        <v>BERICHT</v>
+        <v>Die vier reservierten Bytes dieses Tags sind nicht alle null.</v>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="str">
-        <v>FAIL</v>
+        <v>REPORT</v>
       </c>
       <c r="B442" t="str">
-        <v>FEHLGESCHLAGEN</v>
+        <v>BERICHT</v>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="str">
-        <v>checks</v>
+        <v>FAIL</v>
       </c>
       <c r="B443" t="str">
-        <v>Prüfungen</v>
+        <v>FEHLGESCHLAGEN</v>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="str">
-        <v>Generated by iccPawgReport (iccDEV) · ICC Profile Assessment Working Group checklist.</v>
+        <v>checks</v>
       </c>
       <c r="B444" t="str">
-        <v>Erstellt von iccPawgReport (iccDEV) · Checkliste der ICC Profile Assessment Working Group.</v>
+        <v>Prüfungen</v>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="str">
-        <v>ICC Profile Tool · powered by IccProfLib</v>
+        <v>Generated by iccPawgReport (iccDEV) · ICC Profile Assessment Working Group checklist.</v>
       </c>
       <c r="B445" t="str">
-        <v>ICC-Profil-Tool · betrieben mit IccProfLib</v>
+        <v>Erstellt von iccPawgReport (iccDEV) · Checkliste der ICC Profile Assessment Working Group.</v>
       </c>
     </row>
     <row r="446">
       <c r="A446" t="str">
-        <v>ICC Profile Tool</v>
+        <v>ICC Profile Tool · powered by IccProfLib</v>
       </c>
       <c r="B446" t="str">
-        <v>ICC-Profil-Tool</v>
+        <v>ICC-Profil-Tool · betrieben mit IccProfLib</v>
       </c>
     </row>
     <row r="447">
       <c r="A447" t="str">
-        <v>Powered by {lib}</v>
+        <v>ICC Profile Tool</v>
       </c>
       <c r="B447" t="str">
-        <v>Betrieben mit {lib}</v>
+        <v>ICC-Profil-Tool</v>
       </c>
     </row>
     <row r="448">
       <c r="A448" t="str">
-        <v>Subscribe</v>
+        <v>Powered by {lib}</v>
       </c>
       <c r="B448" t="str">
-        <v>Abonnieren</v>
+        <v>Betrieben mit {lib}</v>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="str">
-        <v>Get notified about new profiletool releases</v>
+        <v>Subscribe</v>
       </c>
       <c r="B449" t="str">
-        <v>Bei neuen profiletool-Releases benachrichtigt werden</v>
+        <v>Abonnieren</v>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="str">
-        <v>Get notified about new releases</v>
+        <v>Get notified about new profiletool releases</v>
       </c>
       <c r="B450" t="str">
-        <v>Bei neuen Releases benachrichtigt werden</v>
+        <v>Bei neuen profiletool-Releases benachrichtigt werden</v>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="str">
-        <v>Close</v>
+        <v>Get notified about new releases</v>
       </c>
       <c r="B451" t="str">
-        <v>Schließen</v>
+        <v>Bei neuen Releases benachrichtigt werden</v>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="str">
-        <v>We’ll email you when a new major or minor profiletool release ships. Patch releases are skipped. Your address is reviewed manually before being added.</v>
+        <v>Close</v>
       </c>
       <c r="B452" t="str">
-        <v>Wir benachrichtigen Sie per E-Mail, sobald ein neues Major- oder Minor-Release von profiletool erscheint. Patch-Releases werden übersprungen. Ihre Adresse wird manuell geprüft, bevor sie aufgenommen wird.</v>
+        <v>Schließen</v>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="str">
-        <v>Email address</v>
+        <v>We’ll email you when a new major or minor profiletool release ships. Patch releases are skipped. Your address is reviewed manually before being added.</v>
       </c>
       <c r="B453" t="str">
-        <v>E-Mail-Adresse</v>
+        <v>Wir benachrichtigen Sie per E-Mail, sobald ein neues Major- oder Minor-Release von profiletool erscheint. Patch-Releases werden übersprungen. Ihre Adresse wird manuell geprüft, bevor sie aufgenommen wird.</v>
       </c>
     </row>
     <row r="454">
       <c r="A454" t="str">
-        <v>you@example.com</v>
+        <v>Email address</v>
       </c>
       <c r="B454" t="str">
-        <v>sie@example.com</v>
+        <v>E-Mail-Adresse</v>
       </c>
     </row>
     <row r="455">
       <c r="A455" t="str">
-        <v>How will you use profiletool?</v>
+        <v>you@example.com</v>
       </c>
       <c r="B455" t="str">
-        <v>Wofür werden Sie profiletool nutzen?</v>
+        <v>sie@example.com</v>
       </c>
     </row>
     <row r="456">
       <c r="A456" t="str">
-        <v>(optional)</v>
+        <v>How will you use profiletool?</v>
       </c>
       <c r="B456" t="str">
-        <v>(optional)</v>
+        <v>Wofür werden Sie profiletool nutzen?</v>
       </c>
     </row>
     <row r="457">
       <c r="A457" t="str">
-        <v>e.g. evaluating ICC profiles for press calibration</v>
+        <v>(optional)</v>
       </c>
       <c r="B457" t="str">
-        <v>z. B. ICC-Profile für Druckkalibrierung evaluieren</v>
+        <v>(optional)</v>
       </c>
     </row>
     <row r="458">
       <c r="A458" t="str">
-        <v>I agree to receive emails about profiletool releases. I can unsubscribe at any time.</v>
+        <v>e.g. evaluating ICC profiles for press calibration</v>
       </c>
       <c r="B458" t="str">
-        <v>Ich willige ein, E-Mails über profiletool-Releases zu erhalten. Ich kann mich jederzeit abmelden.</v>
+        <v>z. B. ICC-Profile für Druckkalibrierung evaluieren</v>
       </c>
     </row>
     <row r="459">
       <c r="A459" t="str">
-        <v>Cancel</v>
+        <v>I agree to receive emails about profiletool releases. I can unsubscribe at any time.</v>
       </c>
       <c r="B459" t="str">
-        <v>Abbrechen</v>
+        <v>Ich willige ein, E-Mails über profiletool-Releases zu erhalten. Ich kann mich jederzeit abmelden.</v>
       </c>
     </row>
     <row r="460">
       <c r="A460" t="str">
-        <v>Subscribe</v>
+        <v>Cancel</v>
       </c>
       <c r="B460" t="str">
-        <v>Abonnieren</v>
+        <v>Abbrechen</v>
       </c>
     </row>
     <row r="461">
       <c r="A461" t="str">
-        <v>Thanks — we’ll be in touch.</v>
+        <v>Subscribe</v>
       </c>
       <c r="B461" t="str">
-        <v>Danke — wir melden uns.</v>
+        <v>Abonnieren</v>
       </c>
     </row>
     <row r="462">
       <c r="A462" t="str">
-        <v>Once approved you’ll receive a welcome email. After that, you’ll only hear from us when a new profiletool release ships.</v>
+        <v>Thanks — we’ll be in touch.</v>
       </c>
       <c r="B462" t="str">
-        <v>Nach Freigabe erhalten Sie eine Willkommens-E-Mail. Danach hören Sie nur dann von uns, wenn ein neues profiletool-Release erscheint.</v>
+        <v>Danke — wir melden uns.</v>
       </c>
     </row>
     <row r="463">
       <c r="A463" t="str">
-        <v>Close</v>
+        <v>Once approved you’ll receive a welcome email. After that, you’ll only hear from us when a new profiletool release ships.</v>
       </c>
       <c r="B463" t="str">
-        <v>Schließen</v>
+        <v>Nach Freigabe erhalten Sie eine Willkommens-E-Mail. Danach hören Sie nur dann von uns, wenn ein neues profiletool-Release erscheint.</v>
       </c>
     </row>
     <row r="464">
       <c r="A464" t="str">
-        <v>Privacy notice</v>
+        <v>Close</v>
       </c>
       <c r="B464" t="str">
-        <v>Datenschutzhinweis</v>
+        <v>Schließen</v>
       </c>
     </row>
     <row r="465">
       <c r="A465" t="str">
-        <v>Please enter a valid email address.</v>
+        <v>Privacy notice</v>
       </c>
       <c r="B465" t="str">
-        <v>Bitte geben Sie eine gültige E-Mail-Adresse ein.</v>
+        <v>Datenschutzhinweis</v>
       </c>
     </row>
     <row r="466">
       <c r="A466" t="str">
-        <v>Too many requests. Please try again later.</v>
+        <v>Please enter a valid email address.</v>
       </c>
       <c r="B466" t="str">
-        <v>Zu viele Anfragen. Bitte versuchen Sie es später erneut.</v>
+        <v>Bitte geben Sie eine gültige E-Mail-Adresse ein.</v>
       </c>
     </row>
     <row r="467">
       <c r="A467" t="str">
-        <v>Please check the form and try again.</v>
+        <v>Too many requests. Please try again later.</v>
       </c>
       <c r="B467" t="str">
-        <v>Bitte überprüfen Sie das Formular und versuchen Sie es erneut.</v>
+        <v>Zu viele Anfragen. Bitte versuchen Sie es später erneut.</v>
       </c>
     </row>
     <row r="468">
       <c r="A468" t="str">
-        <v>Could not send your request. Please try again.</v>
+        <v>Please check the form and try again.</v>
       </c>
       <c r="B468" t="str">
-        <v>Anfrage konnte nicht gesendet werden. Bitte versuchen Sie es erneut.</v>
+        <v>Bitte überprüfen Sie das Formular und versuchen Sie es erneut.</v>
       </c>
     </row>
     <row r="469">
       <c r="A469" t="str">
-        <v>Network error. Please try again.</v>
+        <v>Could not send your request. Please try again.</v>
       </c>
       <c r="B469" t="str">
-        <v>Netzwerkfehler. Bitte versuchen Sie es erneut.</v>
+        <v>Anfrage konnte nicht gesendet werden. Bitte versuchen Sie es erneut.</v>
       </c>
     </row>
     <row r="470">
       <c r="A470" t="str">
-        <v>Error:</v>
+        <v>Network error. Please try again.</v>
       </c>
       <c r="B470" t="str">
-        <v>Fehler:</v>
+        <v>Netzwerkfehler. Bitte versuchen Sie es erneut.</v>
       </c>
     </row>
     <row r="471">
       <c r="A471" t="str">
-        <v>Convert to XML</v>
+        <v>Error:</v>
       </c>
       <c r="B471" t="str">
-        <v>In XML konvertieren</v>
+        <v>Fehler:</v>
       </c>
     </row>
     <row r="472">
       <c r="A472" t="str">
-        <v>Convert to JSON</v>
+        <v>Convert to XML</v>
       </c>
       <c r="B472" t="str">
-        <v>In JSON konvertieren</v>
+        <v>In XML konvertieren</v>
       </c>
     </row>
     <row r="473">
       <c r="A473" t="str">
-        <v>Convert to ICC</v>
+        <v>Convert to JSON</v>
       </c>
       <c r="B473" t="str">
-        <v>In ICC konvertieren</v>
+        <v>In JSON konvertieren</v>
       </c>
     </row>
     <row r="474">
       <c r="A474" t="str">
-        <v>Converting to XML…</v>
+        <v>Convert to ICC</v>
       </c>
       <c r="B474" t="str">
-        <v>Konvertiere in XML…</v>
+        <v>In ICC konvertieren</v>
       </c>
     </row>
     <row r="475">
       <c r="A475" t="str">
-        <v>Converting to JSON…</v>
+        <v>Converting to XML…</v>
       </c>
       <c r="B475" t="str">
-        <v>Konvertiere in JSON…</v>
+        <v>Konvertiere in XML…</v>
       </c>
     </row>
     <row r="476">
       <c r="A476" t="str">
-        <v>Converting to ICC…</v>
+        <v>Converting to JSON…</v>
       </c>
       <c r="B476" t="str">
-        <v>Konvertiere in ICC…</v>
+        <v>Konvertiere in JSON…</v>
       </c>
     </row>
     <row r="477">
       <c r="A477" t="str">
-        <v>Load ICC profile</v>
+        <v>Converting to ICC…</v>
       </c>
       <c r="B477" t="str">
-        <v>ICC-Profil laden</v>
+        <v>Konvertiere in ICC…</v>
       </c>
     </row>
     <row r="478">
       <c r="A478" t="str">
-        <v>Drop zone for ICC profile files</v>
+        <v>Load ICC profile</v>
       </c>
       <c r="B478" t="str">
-        <v>Ablagebereich für ICC-Profil-Dateien</v>
+        <v>ICC-Profil laden</v>
       </c>
     </row>
     <row r="479">
       <c r="A479" t="str">
-        <v>Profile ID</v>
+        <v>Drop zone for ICC profile files</v>
       </c>
       <c r="B479" t="str">
-        <v>Profil-ID</v>
+        <v>Ablagebereich für ICC-Profil-Dateien</v>
       </c>
     </row>
     <row r="480">
       <c r="A480" t="str">
-        <v>No tags found.</v>
+        <v>Profile ID</v>
       </c>
       <c r="B480" t="str">
-        <v>Keine Tags gefunden.</v>
+        <v>Profil-ID</v>
       </c>
     </row>
     <row r="481">
       <c r="A481" t="str">
-        <v>Tag Name</v>
+        <v>No tags found.</v>
       </c>
       <c r="B481" t="str">
-        <v>Tag-Name</v>
+        <v>Keine Tags gefunden.</v>
       </c>
     </row>
     <row r="482">
       <c r="A482" t="str">
-        <v>ID</v>
+        <v>Tag Name</v>
       </c>
       <c r="B482" t="str">
-        <v>ID</v>
+        <v>Tag-Name</v>
       </c>
     </row>
     <row r="483">
       <c r="A483" t="str">
-        <v>Offset</v>
+        <v>ID</v>
       </c>
       <c r="B483" t="str">
-        <v>Offset</v>
+        <v>ID</v>
       </c>
     </row>
     <row r="484">
       <c r="A484" t="str">
-        <v>Size</v>
+        <v>Offset</v>
       </c>
       <c r="B484" t="str">
-        <v>Größe</v>
+        <v>Offset</v>
       </c>
     </row>
     <row r="485">
       <c r="A485" t="str">
-        <v>Pad</v>
+        <v>Size</v>
       </c>
       <c r="B485" t="str">
-        <v>Auffüllung</v>
+        <v>Größe</v>
       </c>
     </row>
     <row r="486">
       <c r="A486" t="str">
-        <v>Bytes changed since load</v>
+        <v>Pad</v>
       </c>
       <c r="B486" t="str">
-        <v>Bytes seit dem Laden geändert</v>
+        <v>Auffüllung</v>
       </c>
     </row>
     <row r="487">
       <c r="A487" t="str">
-        <v>Type</v>
+        <v>Bytes changed since load</v>
       </c>
       <c r="B487" t="str">
-        <v>Typ</v>
+        <v>Bytes seit dem Laden geändert</v>
       </c>
     </row>
     <row r="488">
       <c r="A488" t="str">
-        <v>Array of {type}</v>
+        <v>Type</v>
       </c>
       <c r="B488" t="str">
-        <v>Array von {type}</v>
+        <v>Typ</v>
       </c>
     </row>
     <row r="489">
       <c r="A489" t="str">
-        <v>(No content)</v>
+        <v>Array of {type}</v>
       </c>
       <c r="B489" t="str">
-        <v>(Kein Inhalt)</v>
+        <v>Array von {type}</v>
       </c>
     </row>
     <row r="490">
       <c r="A490" t="str">
-        <v>bytes</v>
+        <v>(No content)</v>
       </c>
       <c r="B490" t="str">
-        <v>Bytes</v>
+        <v>(Kein Inhalt)</v>
       </c>
     </row>
     <row r="491">
       <c r="A491" t="str">
-        <v>Loading full description…</v>
+        <v>bytes</v>
       </c>
       <c r="B491" t="str">
-        <v>Lade vollständige Beschreibung…</v>
+        <v>Bytes</v>
       </c>
     </row>
     <row r="492">
       <c r="A492" t="str">
-        <v>Could not load full description:</v>
+        <v>Loading full description…</v>
       </c>
       <c r="B492" t="str">
-        <v>Vollständige Beschreibung konnte nicht geladen werden:</v>
+        <v>Lade vollständige Beschreibung…</v>
       </c>
     </row>
     <row r="493">
       <c r="A493" t="str">
-        <v>This profile could not be fully parsed and must not be applied. The header and tag directory below are shown for inspection only.</v>
+        <v>Could not load full description:</v>
       </c>
       <c r="B493" t="str">
-        <v>Dieses Profil konnte nicht vollständig gelesen werden und darf nicht angewendet werden. Der Header und das Tag-Verzeichnis unten dienen nur zur Ansicht.</v>
+        <v>Vollständige Beschreibung konnte nicht geladen werden:</v>
       </c>
     </row>
     <row r="494">
       <c r="A494" t="str">
-        <v>Tag contents unavailable — the profile could not be fully parsed.</v>
+        <v>This profile could not be fully parsed and must not be applied. The header and tag directory below are shown for inspection only.</v>
       </c>
       <c r="B494" t="str">
-        <v>Tag-Inhalt nicht verfügbar — das Profil konnte nicht vollständig gelesen werden.</v>
+        <v>Dieses Profil konnte nicht vollständig gelesen werden und darf nicht angewendet werden. Der Header und das Tag-Verzeichnis unten dienen nur zur Ansicht.</v>
       </c>
     </row>
     <row r="495">
       <c r="A495" t="str">
-        <v>No validation output</v>
+        <v>Tag contents unavailable — the profile could not be fully parsed.</v>
       </c>
       <c r="B495" t="str">
-        <v>Keine Validierungsausgabe</v>
+        <v>Tag-Inhalt nicht verfügbar — das Profil konnte nicht vollständig gelesen werden.</v>
       </c>
     </row>
     <row r="496">
       <c r="A496" t="str">
-        <v>Profile is valid</v>
+        <v>No validation output</v>
       </c>
       <c r="B496" t="str">
-        <v>Profil ist gültig</v>
+        <v>Keine Validierungsausgabe</v>
       </c>
     </row>
     <row r="497">
       <c r="A497" t="str">
-        <v>Profile has warning(s)</v>
+        <v>Profile is valid</v>
       </c>
       <c r="B497" t="str">
-        <v>Profil hat Warnung(en)</v>
+        <v>Profil ist gültig</v>
       </c>
     </row>
     <row r="498">
       <c r="A498" t="str">
-        <v>Profile is non-compliant</v>
+        <v>Profile has warning(s)</v>
       </c>
       <c r="B498" t="str">
-        <v>Profil ist nicht konform</v>
+        <v>Profil hat Warnung(en)</v>
       </c>
     </row>
     <row r="499">
       <c r="A499" t="str">
-        <v>Critical validation error</v>
+        <v>Profile is non-compliant</v>
       </c>
       <c r="B499" t="str">
-        <v>Kritischer Validierungsfehler</v>
+        <v>Profil ist nicht konform</v>
       </c>
     </row>
     <row r="500">
       <c r="A500" t="str">
-        <v>Unknown validation status</v>
+        <v>Critical validation error</v>
       </c>
       <c r="B500" t="str">
-        <v>Unbekannter Validierungsstatus</v>
+        <v>Kritischer Validierungsfehler</v>
       </c>
     </row>
     <row r="501">
       <c r="A501" t="str">
-        <v>Critical — shown for inspection only</v>
+        <v>Unknown validation status</v>
       </c>
       <c r="B501" t="str">
-        <v>Kritisch — nur zur Ansicht angezeigt</v>
+        <v>Unbekannter Validierungsstatus</v>
       </c>
     </row>
     <row r="502">
       <c r="A502" t="str">
-        <v>No warnings or errors found.</v>
+        <v>Critical — shown for inspection only</v>
       </c>
       <c r="B502" t="str">
-        <v>Keine Warnungen oder Fehler gefunden.</v>
+        <v>Kritisch — nur zur Ansicht angezeigt</v>
       </c>
     </row>
     <row r="503">
       <c r="A503" t="str">
-        <v>Valid</v>
+        <v>No warnings or errors found.</v>
       </c>
       <c r="B503" t="str">
-        <v>Gültig</v>
+        <v>Keine Warnungen oder Fehler gefunden.</v>
       </c>
     </row>
     <row r="504">
       <c r="A504" t="str">
-        <v>Warning</v>
+        <v>Valid</v>
       </c>
       <c r="B504" t="str">
-        <v>Warnung</v>
+        <v>Gültig</v>
       </c>
     </row>
     <row r="505">
       <c r="A505" t="str">
-        <v>Error</v>
+        <v>Warning</v>
       </c>
       <c r="B505" t="str">
-        <v>Fehler</v>
+        <v>Warnung</v>
       </c>
     </row>
     <row r="506">
       <c r="A506" t="str">
-        <v>Unknown</v>
+        <v>Error</v>
       </c>
       <c r="B506" t="str">
-        <v>Unbekannt</v>
+        <v>Fehler</v>
       </c>
     </row>
     <row r="507">
       <c r="A507" t="str">
-        <v>Pass</v>
+        <v>Unknown</v>
       </c>
       <c r="B507" t="str">
-        <v>Bestanden</v>
+        <v>Unbekannt</v>
       </c>
     </row>
     <row r="508">
       <c r="A508" t="str">
-        <v>Fail</v>
+        <v>Pass</v>
       </c>
       <c r="B508" t="str">
-        <v>Fehlgeschlagen</v>
+        <v>Bestanden</v>
       </c>
     </row>
     <row r="509">
       <c r="A509" t="str">
-        <v>View in context</v>
+        <v>Fail</v>
       </c>
       <c r="B509" t="str">
-        <v>Im Kontext anzeigen</v>
+        <v>Fehlgeschlagen</v>
       </c>
     </row>
     <row r="510">
       <c r="A510" t="str">
-        <v>Validation detail</v>
+        <v>View in context</v>
       </c>
       <c r="B510" t="str">
-        <v>Validierungsdetail</v>
+        <v>Im Kontext anzeigen</v>
       </c>
     </row>
     <row r="511">
       <c r="A511" t="str">
-        <v>Triggered by</v>
+        <v>Validation detail</v>
       </c>
       <c r="B511" t="str">
-        <v>Ausgelöst durch</v>
+        <v>Validierungsdetail</v>
       </c>
     </row>
     <row r="512">
       <c r="A512" t="str">
-        <v>Field</v>
+        <v>Triggered by</v>
       </c>
       <c r="B512" t="str">
-        <v>Feld</v>
+        <v>Ausgelöst durch</v>
       </c>
     </row>
     <row r="513">
       <c r="A513" t="str">
-        <v>Current value</v>
+        <v>Field</v>
       </c>
       <c r="B513" t="str">
-        <v>Aktueller Wert</v>
+        <v>Feld</v>
       </c>
     </row>
     <row r="514">
       <c r="A514" t="str">
-        <v>Required: 0</v>
+        <v>Current value</v>
       </c>
       <c r="B514" t="str">
-        <v>Erforderlich: 0</v>
+        <v>Aktueller Wert</v>
       </c>
     </row>
     <row r="515">
       <c r="A515" t="str">
-        <v>Expected: {value}</v>
+        <v>Required: 0</v>
       </c>
       <c r="B515" t="str">
-        <v>Erwartet: {value}</v>
+        <v>Erforderlich: 0</v>
       </c>
     </row>
     <row r="516">
       <c r="A516" t="str">
-        <v>Invalid</v>
+        <v>Expected: {value}</v>
       </c>
       <c r="B516" t="str">
-        <v>Ungültig</v>
+        <v>Erwartet: {value}</v>
       </c>
     </row>
     <row r="517">
       <c r="A517" t="str">
-        <v>This finding couldn't be tied to a specific field.</v>
+        <v>Invalid</v>
       </c>
       <c r="B517" t="str">
-        <v>Dieser Befund konnte keinem bestimmten Feld zugeordnet werden.</v>
+        <v>Ungültig</v>
       </c>
     </row>
     <row r="518">
       <c r="A518" t="str">
-        <v>Close</v>
+        <v>This finding couldn't be tied to a specific field.</v>
       </c>
       <c r="B518" t="str">
-        <v>Schließen</v>
+        <v>Dieser Befund konnte keinem bestimmten Feld zugeordnet werden.</v>
       </c>
     </row>
     <row r="519">
       <c r="A519" t="str">
-        <v>Loading XML editor…</v>
+        <v>Close</v>
       </c>
       <c r="B519" t="str">
-        <v>Lade XML-Editor…</v>
+        <v>Schließen</v>
       </c>
     </row>
     <row r="520">
       <c r="A520" t="str">
-        <v>Loading JSON editor…</v>
+        <v>Loading XML editor…</v>
       </c>
       <c r="B520" t="str">
-        <v>Lade JSON-Editor…</v>
+        <v>Lade XML-Editor…</v>
       </c>
     </row>
     <row r="521">
       <c r="A521" t="str">
-        <v>You have unsaved XML edits. Overwrite them with a fresh conversion from the ICC profile?</v>
+        <v>Loading JSON editor…</v>
       </c>
       <c r="B521" t="str">
-        <v>Sie haben nicht gespeicherte XML-Änderungen. Mit einer neuen Konvertierung aus dem ICC-Profil überschreiben?</v>
+        <v>Lade JSON-Editor…</v>
       </c>
     </row>
     <row r="522">
       <c r="A522" t="str">
-        <v>You have unsaved JSON edits. Overwrite them with a fresh conversion from the ICC profile?</v>
+        <v>You have unsaved XML edits. Overwrite them with a fresh conversion from the ICC profile?</v>
       </c>
       <c r="B522" t="str">
-        <v>Sie haben nicht gespeicherte JSON-Änderungen. Mit einer neuen Konvertierung aus dem ICC-Profil überschreiben?</v>
+        <v>Sie haben nicht gespeicherte XML-Änderungen. Mit einer neuen Konvertierung aus dem ICC-Profil überschreiben?</v>
       </c>
     </row>
     <row r="523">
       <c r="A523" t="str">
-        <v>● unsaved XML edits</v>
+        <v>You have unsaved JSON edits. Overwrite them with a fresh conversion from the ICC profile?</v>
       </c>
       <c r="B523" t="str">
-        <v>● nicht gespeicherte XML-Änderungen</v>
+        <v>Sie haben nicht gespeicherte JSON-Änderungen. Mit einer neuen Konvertierung aus dem ICC-Profil überschreiben?</v>
       </c>
     </row>
     <row r="524">
       <c r="A524" t="str">
-        <v>● unsaved JSON edits</v>
+        <v>● unsaved XML edits</v>
       </c>
       <c r="B524" t="str">
-        <v>● nicht gespeicherte JSON-Änderungen</v>
+        <v>● nicht gespeicherte XML-Änderungen</v>
       </c>
     </row>
     <row r="525">
       <c r="A525" t="str">
-        <v>Click &lt;em&gt;Convert to XML&lt;/em&gt; to generate an editable XML representation of this profile. The XML is produced by the same IccLibXML code path used by the upstream &lt;code&gt;IccToXml&lt;/code&gt; tool.</v>
+        <v>● unsaved JSON edits</v>
       </c>
       <c r="B525" t="str">
-        <v>Klicken Sie auf &lt;em&gt;In XML konvertieren&lt;/em&gt;, um eine bearbeitbare XML-Darstellung dieses Profils zu erzeugen. Das XML wird vom gleichen IccLibXML-Codepfad erzeugt, den auch das Upstream-Tool &lt;code&gt;IccToXml&lt;/code&gt; verwendet.</v>
+        <v>● nicht gespeicherte JSON-Änderungen</v>
       </c>
     </row>
     <row r="526">
       <c r="A526" t="str">
-        <v>Click &lt;em&gt;Convert to JSON&lt;/em&gt; to generate an editable JSON representation of this profile. The JSON is produced by the same IccLibJSON code path used by the upstream &lt;code&gt;IccToJson&lt;/code&gt; tool.</v>
+        <v>Click &lt;em&gt;Convert to XML&lt;/em&gt; to generate an editable XML representation of this profile. The XML is produced by the same IccLibXML code path used by the upstream &lt;code&gt;IccToXml&lt;/code&gt; tool.</v>
       </c>
       <c r="B526" t="str">
-        <v>Klicken Sie auf &lt;em&gt;In JSON konvertieren&lt;/em&gt;, um eine bearbeitbare JSON-Darstellung dieses Profils zu erzeugen. Das JSON wird vom gleichen IccLibJSON-Codepfad erzeugt, den auch das Upstream-Tool &lt;code&gt;IccToJson&lt;/code&gt; verwendet.</v>
+        <v>Klicken Sie auf &lt;em&gt;In XML konvertieren&lt;/em&gt;, um eine bearbeitbare XML-Darstellung dieses Profils zu erzeugen. Das XML wird vom gleichen IccLibXML-Codepfad erzeugt, den auch das Upstream-Tool &lt;code&gt;IccToXml&lt;/code&gt; verwendet.</v>
       </c>
     </row>
     <row r="527">
       <c r="A527" t="str">
-        <v>indent</v>
+        <v>Click &lt;em&gt;Convert to JSON&lt;/em&gt; to generate an editable JSON representation of this profile. The JSON is produced by the same IccLibJSON code path used by the upstream &lt;code&gt;IccToJson&lt;/code&gt; tool.</v>
       </c>
       <c r="B527" t="str">
-        <v>Einrückung</v>
+        <v>Klicken Sie auf &lt;em&gt;In JSON konvertieren&lt;/em&gt;, um eine bearbeitbare JSON-Darstellung dieses Profils zu erzeugen. Das JSON wird vom gleichen IccLibJSON-Codepfad erzeugt, den auch das Upstream-Tool &lt;code&gt;IccToJson&lt;/code&gt; verwendet.</v>
       </c>
     </row>
     <row r="528">
       <c r="A528" t="str">
-        <v>sort keys</v>
+        <v>indent</v>
       </c>
       <c r="B528" t="str">
-        <v>Schlüssel sortieren</v>
+        <v>Einrückung</v>
       </c>
     </row>
     <row r="529">
       <c r="A529" t="str">
+        <v>sort keys</v>
+      </c>
+      <c r="B529" t="str">
+        <v>Schlüssel sortieren</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="str">
         <v>Profile written from edits, but re-validation failed:</v>
       </c>
-      <c r="B529" t="str">
+      <c r="B530" t="str">
         <v>Profil aus Änderungen geschrieben, aber Neuvalidierung fehlgeschlagen:</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B529"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B530"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
HDR tab: accept JPEG XL files (shown by the browser where it decodes them)
- File picker accepts .jxl; the drop-zone format list says "HEIC and JPEG XL on Safari" in all
  12 locales (xlsx synced).
- Routing is unchanged: JPEG XL is sniffed (FF 0A codestream or the JXL container box) and goes
  to the browser route where the browser decodes it (Safari), and is refused with its reason
  elsewhere; its Inspect capability stays false (profile compressed in the codestream).
- MANUAL HDR tab table and Fit-to-display table name JPEG XL alongside HEIC.

Browser: hdr-review-ui 11/11 (new: picker accepts .jxl), hdr-tab 38/38.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KyeyuyKaCpLNbSR2GQQh3Q
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -3827,10 +3827,10 @@
     </row>
     <row r="428">
       <c r="A428" t="str">
-        <v>OpenEXR, Radiance HDR (.hdr), AVIF, JPEG (including gain-map JPEG), PNG — and HEIC on Safari.</v>
+        <v>OpenEXR, Radiance HDR (.hdr), AVIF, JPEG (including gain-map JPEG), PNG — and HEIC and JPEG XL on Safari.</v>
       </c>
       <c r="B428" t="str">
-        <v>OpenEXR, Radiance HDR (.hdr), AVIF, JPEG (auch Gain-Map-JPEG), PNG – und HEIC in Safari.</v>
+        <v>OpenEXR, Radiance HDR (.hdr), AVIF, JPEG (auch Gain-Map-JPEG), PNG – und HEIC und JPEG XL in Safari.</v>
       </c>
     </row>
     <row r="429">

</xml_diff>